<commit_message>
fix: rebuild batch2 review sheet with all mentor-requested columns
Adds the 'tagged' yes/no column (his first email) alongside norm_tag (the
[#norm:NAME], his second email). Full column set now: line_number, tagged,
norm_tag, refers_to_csr_field_value, refers_to_warl, in_intro_section,
cross_chapter_dup, plus possible_dup. 22 rows (9 new + 13 flagged dups).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/param_extraction/data/batch2_for_review.xlsx
+++ b/param_extraction/data/batch2_for_review.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="batch2" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'batch2'!$A$1:$K$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'batch2'!$A$1:$N$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,20 +457,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:N23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="62" customWidth="1" min="10" max="10"/>
-    <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="12" max="12"/>
+    <col width="58" customWidth="1" min="13" max="13"/>
+    <col width="38" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -506,25 +509,40 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>tagged</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>norm_tag</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>refers_to_csr_field_value</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>refers_to_warl</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>in_intro_section</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>cross_chapter_dup</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>excerpt</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>possible_dup</t>
         </is>
@@ -556,21 +574,19 @@
           <t>smctr.adoc</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>327</t>
-        </is>
+      <c r="F2" s="2" t="n">
+        <v>327</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
           <t>norm:ctrdata_sz_acc</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
           <t>yes</t>
@@ -578,10 +594,21 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
           <t>The `ctrdata` register contains metadata for the recorded transfer. This register must be implemented, though all fields within it are optional. Unimplemented fields are read-only 0.</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr"/>
+      <c r="N2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -609,17 +636,15 @@
           <t>hypervisor.adoc</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>430</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+      <c r="F3" s="2" t="n">
+        <v>430</v>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr"/>
       <c r="I3" s="2" t="inlineStr">
         <is>
           <t>yes</t>
@@ -627,10 +652,21 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr"/>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
           <t>If bit _i_ of `sie` is read-only zero, the same bit in register `hip` may be writable or may be read-only.</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr"/>
+      <c r="N3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -658,17 +694,15 @@
           <t>smcdeleg.adoc</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>138</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+      <c r="F4" s="2" t="n">
+        <v>138</v>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
       <c r="I4" s="2" t="inlineStr">
         <is>
           <t>no</t>
@@ -676,10 +710,21 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
           <t>It is optional whether the LCOFI bit (bit 13) in each of mideleg and hideleg, which allows all LCOFIs to be delegated to S-mode and VS-mode, respectively, is implemented and writable.</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr"/>
+      <c r="N4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -707,21 +752,19 @@
           <t>machine.adoc</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>1836</t>
-        </is>
+      <c r="F5" s="2" t="n">
+        <v>1836</v>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
           <t>norm:pma_idp_implicit_sz</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
           <t>no</t>
@@ -729,10 +772,21 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr"/>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
           <t>The size of these naturally aligned power-of-2 regions is implementation-defined, but, for systems with page-based virtual memory, must not exceed the smallest supported page size.</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr"/>
+      <c r="N5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -760,28 +814,37 @@
           <t>supervisor.adoc</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>530</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+      <c r="F6" s="2" t="n">
+        <v>530</v>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
           <t>`sepc` is a *WARL* register that must be able to hold all valid virtual addresses. It need not be capable of holding all possible invalid addresses. Prior to writing `sepc`, implementations may convert an invalid address into some other invalid address that `sepc` is capable of holding.</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr"/>
+      <c r="N6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -809,21 +872,19 @@
           <t>indirect-csr.adoc</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>138</t>
-        </is>
+      <c r="F7" s="2" t="n">
+        <v>138</v>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
           <t>norm:siselect_min_range</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
           <t>no</t>
@@ -831,10 +892,21 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr"/>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
           <t>The `siselect` register will support the value range 0..0xFFF at a minimum. A future extension may define a value range outside of this minimum range. Only if such an extension is implemented will `siselect` be required to support larger values.</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr"/>
+      <c r="N7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -862,21 +934,19 @@
           <t>indirect-csr.adoc</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>213</t>
-        </is>
+      <c r="F8" s="2" t="n">
+        <v>213</v>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
           <t>norm:vsiselect_min_range</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
           <t>no</t>
@@ -884,10 +954,21 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr"/>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
           <t>The `vsiselect` register will support the value range 0..0xFFF at a minimum. A future extension may define a value range outside of this minimum range. Only if such an extension is implemented will `vsiselect` be required to support larger values.</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr"/>
+      <c r="N8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -915,21 +996,19 @@
           <t>machine.adoc</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>1590</t>
-        </is>
+      <c r="F9" s="2" t="n">
+        <v>1590</v>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
           <t>norm:wfi_resume_reason</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
           <t>no</t>
@@ -937,10 +1016,21 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr"/>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
           <t>Implementations are permitted to resume execution for any reason, even if an enabled interrupt has not become pending. Hence, a legal implementation is to simply implement the WFI instruction as a NOP.</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr"/>
+      <c r="N9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -968,17 +1058,15 @@
           <t>zc.adoc</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>1121</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+      <c r="F10" s="2" t="n">
+        <v>1121</v>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
       <c r="I10" s="2" t="inlineStr">
         <is>
           <t>no</t>
@@ -986,10 +1074,21 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
           <t>It is platform defined whether the core implementation waits for the bus responses before continuing to the final stage of the sequence, or handles errors responses after completing the PUSH instruction.</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr"/>
+      <c r="N10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -1017,28 +1116,37 @@
           <t>hypervisor.adoc</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>627</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="inlineStr"/>
-      <c r="H11" s="3" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+      <c r="F11" s="3" t="n">
+        <v>627</v>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr"/>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L11" s="3" t="inlineStr"/>
+      <c r="M11" s="3" t="inlineStr">
+        <is>
           <t>An implementation that supports only the defined paged virtual-memory schemes and/or Bare may make PPN[1:0] read-only zero.</t>
         </is>
       </c>
-      <c r="K11" s="3" t="inlineStr">
+      <c r="N11" s="3" t="inlineStr">
         <is>
           <t>HGATP_PPN_LOWER_BITS_RO (sent, V4)</t>
         </is>
@@ -1070,28 +1178,37 @@
           <t>smcdeleg.adoc</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>63</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr"/>
-      <c r="H12" s="3" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+      <c r="F12" s="3" t="n">
+        <v>63</v>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr"/>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L12" s="3" t="inlineStr"/>
+      <c r="M12" s="3" t="inlineStr">
+        <is>
           <t>hpmevent__i__ may represent a subset of the state accessed by the mhpmevent__i__ register. Specifically, if Sscofpmf is implemented, event selector bit 62 (MINH) is read-only 0 when accessed through sireg*.</t>
         </is>
       </c>
-      <c r="K12" s="3" t="inlineStr">
+      <c r="N12" s="3" t="inlineStr">
         <is>
           <t>HPMEVENT_SUBSET_REPRESENTATION (sent, borderline)</t>
         </is>
@@ -1123,21 +1240,19 @@
           <t>machine.adoc</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>952</t>
-        </is>
+      <c r="F13" s="3" t="n">
+        <v>952</v>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
           <t>norm:medeleg_mideleg_op1</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -1145,10 +1260,21 @@
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L13" s="3" t="inlineStr"/>
+      <c r="M13" s="3" t="inlineStr">
+        <is>
           <t>implementations can provide individual read/write bits within `medeleg` and `mideleg` to indicate that certain exceptions and interrupts should be processed directly by a lower privilege level.</t>
         </is>
       </c>
-      <c r="K13" s="3" t="inlineStr">
+      <c r="N13" s="3" t="inlineStr">
         <is>
           <t>DELEGATABLE_EXCEPTIONS (sent)</t>
         </is>
@@ -1180,32 +1306,41 @@
           <t>machine.adoc</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>975</t>
-        </is>
+      <c r="F14" s="3" t="n">
+        <v>975</v>
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
           <t>norm:medeleg_mideleg_warl</t>
         </is>
       </c>
-      <c r="H14" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L14" s="3" t="inlineStr"/>
+      <c r="M14" s="3" t="inlineStr">
+        <is>
           <t>An implementation can choose to subset the delegatable traps, with the supported delegatable bits found by writing one to every bit location, then reading back the value in `medeleg` or `mideleg` to see which bit positions hold a one.</t>
         </is>
       </c>
-      <c r="K14" s="3" t="inlineStr">
+      <c r="N14" s="3" t="inlineStr">
         <is>
           <t>DELEGATABLE_EXCEPTIONS (sent)</t>
         </is>
@@ -1237,17 +1372,15 @@
           <t>intro.adoc</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>468</t>
-        </is>
-      </c>
-      <c r="G15" s="3" t="inlineStr"/>
-      <c r="H15" s="3" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+      <c r="F15" s="3" t="n">
+        <v>468</v>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr"/>
       <c r="I15" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -1255,10 +1388,21 @@
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="L15" s="3" t="inlineStr"/>
+      <c r="M15" s="3" t="inlineStr">
+        <is>
           <t>Optionally, an implementation may adopt the stronger model of Total Store Ordering, as defined in &lt;&lt;ztso&gt;&gt;.</t>
         </is>
       </c>
-      <c r="K15" s="3" t="inlineStr">
+      <c r="N15" s="3" t="inlineStr">
         <is>
           <t>MEMORY_ORDERING_MODEL=Ztso (sent)</t>
         </is>
@@ -1290,21 +1434,19 @@
           <t>machine.adoc</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>1476</t>
-        </is>
+      <c r="F16" s="3" t="n">
+        <v>1476</v>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
           <t>norm:menvcfg_fiom_rdonly0_ok</t>
         </is>
       </c>
-      <c r="H16" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
           <t>yes</t>
@@ -1312,10 +1454,21 @@
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K16" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L16" s="3" t="inlineStr"/>
+      <c r="M16" s="3" t="inlineStr">
+        <is>
           <t>If S-mode is not supported, or if `satp`.MODE is read-only zero (always Bare), the implementation may make FIOM read-only zero.</t>
         </is>
       </c>
-      <c r="K16" s="3" t="inlineStr">
+      <c r="N16" s="3" t="inlineStr">
         <is>
           <t>MENVCFG_FIOM_READONLY (sent)</t>
         </is>
@@ -1347,21 +1500,19 @@
           <t>machine.adoc</t>
         </is>
       </c>
-      <c r="F17" s="3" t="inlineStr">
-        <is>
-          <t>1083</t>
-        </is>
+      <c r="F17" s="3" t="n">
+        <v>1083</v>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
           <t>norm:mip_msip_mie_msie_maybe_rdonly0</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
           <t>yes</t>
@@ -1369,10 +1520,21 @@
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L17" s="3" t="inlineStr"/>
+      <c r="M17" s="3" t="inlineStr">
+        <is>
           <t>If a system has only one hart, or if a platform standard supports the delivery of machine-level interprocessor interrupts through external interrupts (MEI) instead, then `mip`.MSIP and `mie`.MSIE may both be read-only zeros.</t>
         </is>
       </c>
-      <c r="K17" s="3" t="inlineStr">
+      <c r="N17" s="3" t="inlineStr">
         <is>
           <t>MIP_MSIP_MIE_MSIE_READONLY (sent)</t>
         </is>
@@ -1404,21 +1566,19 @@
           <t>indirect-csr.adoc</t>
         </is>
       </c>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>73</t>
-        </is>
+      <c r="F18" s="3" t="n">
+        <v>73</v>
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
           <t>norm:miselect_min_sz</t>
         </is>
       </c>
-      <c r="H18" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
           <t>yes</t>
@@ -1426,10 +1586,21 @@
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K18" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L18" s="3" t="inlineStr"/>
+      <c r="M18" s="3" t="inlineStr">
+        <is>
           <t>The `miselect` register implements at least enough bits to support all implemented `miselect` values (corresponding to the implemented extensions that utilize `miselect`/`mireg*` to indirectly access register state). The `miselect` register may be read-only zero if there are no extensions implemented that utilize it.</t>
         </is>
       </c>
-      <c r="K18" s="3" t="inlineStr">
+      <c r="N18" s="3" t="inlineStr">
         <is>
           <t>MISELECT_WIDTH (sent, borderline)</t>
         </is>
@@ -1461,28 +1632,37 @@
           <t>scalar-crypto.adoc</t>
         </is>
       </c>
-      <c r="F19" s="3" t="inlineStr">
-        <is>
-          <t>3697</t>
-        </is>
-      </c>
-      <c r="G19" s="3" t="inlineStr"/>
-      <c r="H19" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+      <c r="F19" s="3" t="n">
+        <v>3697</v>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr"/>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K19" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L19" s="3" t="inlineStr"/>
+      <c r="M19" s="3" t="inlineStr">
+        <is>
           <t>Implementations may implement `mseccfg` such that `[s,u]seed` is a read-only constant value `0`.</t>
         </is>
       </c>
-      <c r="K19" s="3" t="inlineStr">
+      <c r="N19" s="3" t="inlineStr">
         <is>
           <t>SSEED_USEED_WRITABLE (sent)</t>
         </is>
@@ -1514,21 +1694,19 @@
           <t>machine.adoc</t>
         </is>
       </c>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>1812</t>
-        </is>
+      <c r="F20" s="3" t="n">
+        <v>1812</v>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
           <t>norm:pma_mag_exc</t>
         </is>
       </c>
-      <c r="H20" s="3" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -1536,10 +1714,21 @@
       </c>
       <c r="J20" s="3" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K20" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L20" s="3" t="inlineStr"/>
+      <c r="M20" s="3" t="inlineStr">
+        <is>
           <t>Implementations may raise access-fault exceptions instead of address-misaligned exceptions for some misaligned accesses, indicating the instruction should not be emulated by a trap handler.</t>
         </is>
       </c>
-      <c r="K20" s="3" t="inlineStr">
+      <c r="N20" s="3" t="inlineStr">
         <is>
           <t>MISALIGNED_LDST_EXCEPTION_PRIORITY (existing UDB)</t>
         </is>
@@ -1571,21 +1760,19 @@
           <t>machine.adoc</t>
         </is>
       </c>
-      <c r="F21" s="3" t="inlineStr">
-        <is>
-          <t>3352</t>
-        </is>
+      <c r="F21" s="3" t="n">
+        <v>3352</v>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
           <t>norm:pmp_mmode_locking</t>
         </is>
       </c>
-      <c r="H21" s="3" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -1593,10 +1780,21 @@
       </c>
       <c r="J21" s="3" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K21" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L21" s="3" t="inlineStr"/>
+      <c r="M21" s="3" t="inlineStr">
+        <is>
           <t>Optionally, PMP checks may additionally apply to M-mode accesses, in which case the PMP registers themselves are locked, so that even M-mode software cannot change them until the hart is reset.</t>
         </is>
       </c>
-      <c r="K21" s="3" t="inlineStr">
+      <c r="N21" s="3" t="inlineStr">
         <is>
           <t>PMP_MMODE_ENFORCEMENT (sent, rejected)</t>
         </is>
@@ -1628,21 +1826,19 @@
           <t>unpriv-cfi.adoc</t>
         </is>
       </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>530</t>
-        </is>
+      <c r="F22" s="3" t="n">
+        <v>530</v>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
           <t>norm:ssp-field_1_0</t>
         </is>
       </c>
-      <c r="H22" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
           <t>yes</t>
@@ -1650,10 +1846,21 @@
       </c>
       <c r="J22" s="3" t="inlineStr">
         <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K22" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L22" s="3" t="inlineStr"/>
+      <c r="M22" s="3" t="inlineStr">
+        <is>
           <t>The bits 1:0 of `ssp` are read-only zero. If the UXLEN or SXLEN may never be 32, then the bit 2 is also read-only zero.</t>
         </is>
       </c>
-      <c r="K22" s="3" t="inlineStr">
+      <c r="N22" s="3" t="inlineStr">
         <is>
           <t>SSP_BIT2 (sent)</t>
         </is>
@@ -1685,17 +1892,15 @@
           <t>machine.adoc</t>
         </is>
       </c>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
-          <t>1572</t>
-        </is>
-      </c>
-      <c r="G23" s="3" t="inlineStr"/>
-      <c r="H23" s="3" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+      <c r="F23" s="3" t="n">
+        <v>1572</v>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr"/>
       <c r="I23" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -1703,17 +1908,28 @@
       </c>
       <c r="J23" s="3" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K23" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L23" s="3" t="inlineStr"/>
+      <c r="M23" s="3" t="inlineStr">
+        <is>
           <t>WFI is available in all privileged modes, and optionally available to U-mode.</t>
         </is>
       </c>
-      <c r="K23" s="3" t="inlineStr">
+      <c r="N23" s="3" t="inlineStr">
         <is>
           <t>WFI_U_MODE (sent, dup)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K23"/>
+  <autoFilter ref="A1:N23"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>